<commit_message>
Add the possibility to import recipients into rubrics from XLSX
</commit_message>
<xml_diff>
--- a/test/assets/xlsx/import_standard.xlsx
+++ b/test/assets/xlsx/import_standard.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="17">
   <si>
     <t xml:space="preserve">DENOMINAZIONE</t>
   </si>
@@ -71,9 +71,6 @@
   </si>
   <si>
     <t xml:space="preserve">Via Testi 50</t>
-  </si>
-  <si>
-    <t xml:space="preserve">09071</t>
   </si>
 </sst>
 </file>
@@ -267,7 +264,7 @@
         <v>14</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>70031</v>
+        <v>76123</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>8</v>
@@ -283,10 +280,12 @@
       <c r="B5" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C5" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D5" s="2"/>
+      <c r="C5" s="2" t="n">
+        <v>76123</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>8</v>
+      </c>
       <c r="E5" s="2"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
(feat): Sender import from XLSX route
</commit_message>
<xml_diff>
--- a/test/assets/xlsx/import_standard.xlsx
+++ b/test/assets/xlsx/import_standard.xlsx
@@ -264,7 +264,7 @@
         <v>14</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>76123</v>
+        <v>70031</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>8</v>
@@ -283,10 +283,10 @@
       <c r="C5" s="2" t="n">
         <v>76123</v>
       </c>
-      <c r="D5" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E5" s="2"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2"/>

</xml_diff>